<commit_message>
daily auto-refresh 2026-08-19 01:59
</commit_message>
<xml_diff>
--- a/no_gmv_data.xlsx
+++ b/no_gmv_data.xlsx
@@ -619,7 +619,11 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
@@ -676,7 +680,7 @@
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>South Asian</t>
+          <t>Black/African</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
@@ -733,7 +737,11 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
@@ -961,7 +969,11 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
@@ -1185,7 +1197,11 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr"/>
@@ -1409,7 +1425,11 @@
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr"/>
@@ -1519,7 +1539,11 @@
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr"/>
@@ -1629,7 +1653,11 @@
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr"/>
@@ -2026,7 +2054,11 @@
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr"/>
@@ -2313,7 +2345,11 @@
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr"/>
@@ -2545,7 +2581,11 @@
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr"/>
@@ -2891,7 +2931,11 @@
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J43" t="inlineStr"/>
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr"/>
@@ -3017,7 +3061,11 @@
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr"/>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J45" t="inlineStr"/>
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr"/>
@@ -3186,7 +3234,11 @@
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr"/>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J48" t="inlineStr"/>
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr"/>
@@ -3469,7 +3521,11 @@
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr"/>
-      <c r="I53" t="inlineStr"/>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J53" t="inlineStr"/>
       <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr"/>
@@ -3634,7 +3690,11 @@
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr"/>
-      <c r="I56" t="inlineStr"/>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J56" t="inlineStr"/>
       <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr"/>
@@ -3703,7 +3763,7 @@
       <c r="H57" t="inlineStr"/>
       <c r="I57" t="inlineStr">
         <is>
-          <t>East/SE Asian</t>
+          <t>Black/African</t>
         </is>
       </c>
       <c r="J57" t="inlineStr"/>
@@ -3760,7 +3820,11 @@
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr"/>
-      <c r="I58" t="inlineStr"/>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J58" t="inlineStr"/>
       <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr"/>
@@ -4204,7 +4268,11 @@
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr"/>
-      <c r="I66" t="inlineStr"/>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Mixed/Ambiguous</t>
+        </is>
+      </c>
       <c r="J66" t="inlineStr"/>
       <c r="K66" t="inlineStr"/>
       <c r="L66" t="inlineStr"/>
@@ -4428,7 +4496,11 @@
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr"/>
       <c r="H70" t="inlineStr"/>
-      <c r="I70" t="inlineStr"/>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J70" t="inlineStr"/>
       <c r="K70" t="inlineStr"/>
       <c r="L70" t="inlineStr"/>
@@ -4939,7 +5011,11 @@
       <c r="F79" t="inlineStr"/>
       <c r="G79" t="inlineStr"/>
       <c r="H79" t="inlineStr"/>
-      <c r="I79" t="inlineStr"/>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J79" t="inlineStr"/>
       <c r="K79" t="inlineStr"/>
       <c r="L79" t="inlineStr"/>
@@ -5108,7 +5184,11 @@
       <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr"/>
-      <c r="I82" t="inlineStr"/>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J82" t="inlineStr"/>
       <c r="K82" t="inlineStr"/>
       <c r="L82" t="inlineStr"/>
@@ -5501,7 +5581,11 @@
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="inlineStr"/>
-      <c r="I89" t="inlineStr"/>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J89" t="inlineStr"/>
       <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr"/>
@@ -5556,7 +5640,11 @@
       <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr"/>
-      <c r="I90" t="inlineStr"/>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J90" t="inlineStr"/>
       <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr"/>
@@ -5611,7 +5699,11 @@
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr"/>
       <c r="H91" t="inlineStr"/>
-      <c r="I91" t="inlineStr"/>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J91" t="inlineStr"/>
       <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr"/>
@@ -5666,7 +5758,11 @@
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr"/>
-      <c r="I92" t="inlineStr"/>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J92" t="inlineStr"/>
       <c r="K92" t="inlineStr"/>
       <c r="L92" t="inlineStr"/>
@@ -5890,7 +5986,11 @@
       <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr"/>
       <c r="H96" t="inlineStr"/>
-      <c r="I96" t="inlineStr"/>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J96" t="inlineStr"/>
       <c r="K96" t="inlineStr"/>
       <c r="L96" t="inlineStr"/>
@@ -6409,7 +6509,11 @@
       <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr"/>
       <c r="H105" t="inlineStr"/>
-      <c r="I105" t="inlineStr"/>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J105" t="inlineStr"/>
       <c r="K105" t="inlineStr"/>
       <c r="L105" t="inlineStr"/>
@@ -6523,7 +6627,11 @@
       <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr"/>
       <c r="H107" t="inlineStr"/>
-      <c r="I107" t="inlineStr"/>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J107" t="inlineStr"/>
       <c r="K107" t="inlineStr"/>
       <c r="L107" t="inlineStr"/>
@@ -6578,7 +6686,11 @@
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr"/>
       <c r="H108" t="inlineStr"/>
-      <c r="I108" t="inlineStr"/>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>South Asian</t>
+        </is>
+      </c>
       <c r="J108" t="inlineStr"/>
       <c r="K108" t="inlineStr"/>
       <c r="L108" t="inlineStr"/>
@@ -6633,7 +6745,11 @@
       <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr"/>
       <c r="H109" t="inlineStr"/>
-      <c r="I109" t="inlineStr"/>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J109" t="inlineStr"/>
       <c r="K109" t="inlineStr"/>
       <c r="L109" t="inlineStr"/>
@@ -6749,7 +6865,7 @@
       <c r="H111" t="inlineStr"/>
       <c r="I111" t="inlineStr">
         <is>
-          <t>White/European</t>
+          <t>Black/African</t>
         </is>
       </c>
       <c r="J111" t="inlineStr"/>
@@ -6981,7 +7097,7 @@
       <c r="H115" t="inlineStr"/>
       <c r="I115" t="inlineStr">
         <is>
-          <t>Hispanic/Latino</t>
+          <t>South Asian</t>
         </is>
       </c>
       <c r="J115" t="inlineStr"/>
@@ -7435,7 +7551,11 @@
       <c r="F123" t="inlineStr"/>
       <c r="G123" t="inlineStr"/>
       <c r="H123" t="inlineStr"/>
-      <c r="I123" t="inlineStr"/>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J123" t="inlineStr"/>
       <c r="K123" t="inlineStr"/>
       <c r="L123" t="inlineStr"/>
@@ -7545,7 +7665,11 @@
       <c r="F125" t="inlineStr"/>
       <c r="G125" t="inlineStr"/>
       <c r="H125" t="inlineStr"/>
-      <c r="I125" t="inlineStr"/>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J125" t="inlineStr"/>
       <c r="K125" t="inlineStr"/>
       <c r="L125" t="inlineStr"/>
@@ -8064,7 +8188,11 @@
       <c r="F134" t="inlineStr"/>
       <c r="G134" t="inlineStr"/>
       <c r="H134" t="inlineStr"/>
-      <c r="I134" t="inlineStr"/>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J134" t="inlineStr"/>
       <c r="K134" t="inlineStr"/>
       <c r="L134" t="inlineStr"/>
@@ -8340,7 +8468,11 @@
       <c r="F138" t="inlineStr"/>
       <c r="G138" t="inlineStr"/>
       <c r="H138" t="inlineStr"/>
-      <c r="I138" t="inlineStr"/>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J138" t="inlineStr"/>
       <c r="K138" t="inlineStr"/>
       <c r="L138" t="inlineStr"/>
@@ -8568,7 +8700,11 @@
       <c r="F142" t="inlineStr"/>
       <c r="G142" t="inlineStr"/>
       <c r="H142" t="inlineStr"/>
-      <c r="I142" t="inlineStr"/>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J142" t="inlineStr"/>
       <c r="K142" t="inlineStr"/>
       <c r="L142" t="inlineStr"/>
@@ -8767,7 +8903,7 @@
       <c r="H145" t="inlineStr"/>
       <c r="I145" t="inlineStr">
         <is>
-          <t>Black/African</t>
+          <t>White/European</t>
         </is>
       </c>
       <c r="J145" t="inlineStr"/>
@@ -8938,7 +9074,11 @@
       <c r="F148" t="inlineStr"/>
       <c r="G148" t="inlineStr"/>
       <c r="H148" t="inlineStr"/>
-      <c r="I148" t="inlineStr"/>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J148" t="inlineStr"/>
       <c r="K148" t="inlineStr"/>
       <c r="L148" t="inlineStr"/>
@@ -9339,7 +9479,11 @@
       <c r="F155" t="inlineStr"/>
       <c r="G155" t="inlineStr"/>
       <c r="H155" t="inlineStr"/>
-      <c r="I155" t="inlineStr"/>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J155" t="inlineStr"/>
       <c r="K155" t="inlineStr"/>
       <c r="L155" t="inlineStr"/>
@@ -9394,7 +9538,11 @@
       <c r="F156" t="inlineStr"/>
       <c r="G156" t="inlineStr"/>
       <c r="H156" t="inlineStr"/>
-      <c r="I156" t="inlineStr"/>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J156" t="inlineStr"/>
       <c r="K156" t="inlineStr"/>
       <c r="L156" t="inlineStr"/>
@@ -9567,7 +9715,11 @@
       <c r="F159" t="inlineStr"/>
       <c r="G159" t="inlineStr"/>
       <c r="H159" t="inlineStr"/>
-      <c r="I159" t="inlineStr"/>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J159" t="inlineStr"/>
       <c r="K159" t="inlineStr"/>
       <c r="L159" t="inlineStr"/>
@@ -9734,7 +9886,7 @@
       <c r="H162" t="inlineStr"/>
       <c r="I162" t="inlineStr">
         <is>
-          <t>White/European</t>
+          <t>Black/African</t>
         </is>
       </c>
       <c r="J162" t="inlineStr"/>
@@ -9793,7 +9945,7 @@
       <c r="H163" t="inlineStr"/>
       <c r="I163" t="inlineStr">
         <is>
-          <t>Black/African</t>
+          <t>Mixed/Ambiguous</t>
         </is>
       </c>
       <c r="J163" t="inlineStr"/>
@@ -9850,7 +10002,11 @@
       <c r="F164" t="inlineStr"/>
       <c r="G164" t="inlineStr"/>
       <c r="H164" t="inlineStr"/>
-      <c r="I164" t="inlineStr"/>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J164" t="inlineStr"/>
       <c r="K164" t="inlineStr"/>
       <c r="L164" t="inlineStr"/>
@@ -10353,7 +10509,11 @@
       <c r="F173" t="inlineStr"/>
       <c r="G173" t="inlineStr"/>
       <c r="H173" t="inlineStr"/>
-      <c r="I173" t="inlineStr"/>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J173" t="inlineStr"/>
       <c r="K173" t="inlineStr"/>
       <c r="L173" t="inlineStr"/>
@@ -10597,7 +10757,11 @@
       <c r="F177" t="inlineStr"/>
       <c r="G177" t="inlineStr"/>
       <c r="H177" t="inlineStr"/>
-      <c r="I177" t="inlineStr"/>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J177" t="inlineStr"/>
       <c r="K177" t="inlineStr"/>
       <c r="L177" t="inlineStr"/>
@@ -10652,7 +10816,11 @@
       <c r="F178" t="inlineStr"/>
       <c r="G178" t="inlineStr"/>
       <c r="H178" t="inlineStr"/>
-      <c r="I178" t="inlineStr"/>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J178" t="inlineStr"/>
       <c r="K178" t="inlineStr"/>
       <c r="L178" t="inlineStr"/>
@@ -10764,7 +10932,7 @@
       <c r="H180" t="inlineStr"/>
       <c r="I180" t="inlineStr">
         <is>
-          <t>White/European</t>
+          <t>Black/African</t>
         </is>
       </c>
       <c r="J180" t="inlineStr"/>
@@ -10876,7 +11044,11 @@
       <c r="F182" t="inlineStr"/>
       <c r="G182" t="inlineStr"/>
       <c r="H182" t="inlineStr"/>
-      <c r="I182" t="inlineStr"/>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>East/SE Asian</t>
+        </is>
+      </c>
       <c r="J182" t="inlineStr"/>
       <c r="K182" t="inlineStr"/>
       <c r="L182" t="inlineStr"/>
@@ -11100,7 +11272,11 @@
       <c r="F186" t="inlineStr"/>
       <c r="G186" t="inlineStr"/>
       <c r="H186" t="inlineStr"/>
-      <c r="I186" t="inlineStr"/>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J186" t="inlineStr"/>
       <c r="K186" t="inlineStr"/>
       <c r="L186" t="inlineStr"/>
@@ -11438,7 +11614,11 @@
       <c r="F192" t="inlineStr"/>
       <c r="G192" t="inlineStr"/>
       <c r="H192" t="inlineStr"/>
-      <c r="I192" t="inlineStr"/>
+      <c r="I192" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J192" t="inlineStr"/>
       <c r="K192" t="inlineStr"/>
       <c r="L192" t="inlineStr"/>
@@ -11717,7 +11897,11 @@
       <c r="F197" t="inlineStr"/>
       <c r="G197" t="inlineStr"/>
       <c r="H197" t="inlineStr"/>
-      <c r="I197" t="inlineStr"/>
+      <c r="I197" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J197" t="inlineStr"/>
       <c r="K197" t="inlineStr"/>
       <c r="L197" t="inlineStr"/>
@@ -11945,7 +12129,11 @@
       <c r="F201" t="inlineStr"/>
       <c r="G201" t="inlineStr"/>
       <c r="H201" t="inlineStr"/>
-      <c r="I201" t="inlineStr"/>
+      <c r="I201" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J201" t="inlineStr"/>
       <c r="K201" t="inlineStr"/>
       <c r="L201" t="inlineStr"/>
@@ -12000,7 +12188,11 @@
       <c r="F202" t="inlineStr"/>
       <c r="G202" t="inlineStr"/>
       <c r="H202" t="inlineStr"/>
-      <c r="I202" t="inlineStr"/>
+      <c r="I202" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J202" t="inlineStr"/>
       <c r="K202" t="inlineStr"/>
       <c r="L202" t="inlineStr"/>
@@ -12456,7 +12648,11 @@
       <c r="F210" t="inlineStr"/>
       <c r="G210" t="inlineStr"/>
       <c r="H210" t="inlineStr"/>
-      <c r="I210" t="inlineStr"/>
+      <c r="I210" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J210" t="inlineStr"/>
       <c r="K210" t="inlineStr"/>
       <c r="L210" t="inlineStr"/>
@@ -12631,7 +12827,7 @@
       <c r="H213" t="inlineStr"/>
       <c r="I213" t="inlineStr">
         <is>
-          <t>Black/African</t>
+          <t>White/European</t>
         </is>
       </c>
       <c r="J213" t="inlineStr"/>
@@ -12690,7 +12886,7 @@
       <c r="H214" t="inlineStr"/>
       <c r="I214" t="inlineStr">
         <is>
-          <t>Middle Eastern/Arab</t>
+          <t>Black/African</t>
         </is>
       </c>
       <c r="J214" t="inlineStr"/>
@@ -12806,7 +13002,11 @@
       <c r="F216" t="inlineStr"/>
       <c r="G216" t="inlineStr"/>
       <c r="H216" t="inlineStr"/>
-      <c r="I216" t="inlineStr"/>
+      <c r="I216" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J216" t="inlineStr"/>
       <c r="K216" t="inlineStr"/>
       <c r="L216" t="inlineStr"/>
@@ -12920,7 +13120,11 @@
       <c r="F218" t="inlineStr"/>
       <c r="G218" t="inlineStr"/>
       <c r="H218" t="inlineStr"/>
-      <c r="I218" t="inlineStr"/>
+      <c r="I218" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J218" t="inlineStr"/>
       <c r="K218" t="inlineStr"/>
       <c r="L218" t="inlineStr"/>
@@ -13030,7 +13234,11 @@
       <c r="F220" t="inlineStr"/>
       <c r="G220" t="inlineStr"/>
       <c r="H220" t="inlineStr"/>
-      <c r="I220" t="inlineStr"/>
+      <c r="I220" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J220" t="inlineStr"/>
       <c r="K220" t="inlineStr"/>
       <c r="L220" t="inlineStr"/>
@@ -13486,7 +13694,11 @@
       <c r="F228" t="inlineStr"/>
       <c r="G228" t="inlineStr"/>
       <c r="H228" t="inlineStr"/>
-      <c r="I228" t="inlineStr"/>
+      <c r="I228" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J228" t="inlineStr"/>
       <c r="K228" t="inlineStr"/>
       <c r="L228" t="inlineStr"/>
@@ -13596,7 +13808,11 @@
       <c r="F230" t="inlineStr"/>
       <c r="G230" t="inlineStr"/>
       <c r="H230" t="inlineStr"/>
-      <c r="I230" t="inlineStr"/>
+      <c r="I230" t="inlineStr">
+        <is>
+          <t>South Asian</t>
+        </is>
+      </c>
       <c r="J230" t="inlineStr"/>
       <c r="K230" t="inlineStr"/>
       <c r="L230" t="inlineStr"/>
@@ -13761,7 +13977,11 @@
       <c r="F233" t="inlineStr"/>
       <c r="G233" t="inlineStr"/>
       <c r="H233" t="inlineStr"/>
-      <c r="I233" t="inlineStr"/>
+      <c r="I233" t="inlineStr">
+        <is>
+          <t>South Asian</t>
+        </is>
+      </c>
       <c r="J233" t="inlineStr"/>
       <c r="K233" t="inlineStr"/>
       <c r="L233" t="inlineStr"/>
@@ -13828,7 +14048,11 @@
       <c r="F234" t="inlineStr"/>
       <c r="G234" t="inlineStr"/>
       <c r="H234" t="inlineStr"/>
-      <c r="I234" t="inlineStr"/>
+      <c r="I234" t="inlineStr">
+        <is>
+          <t>South Asian</t>
+        </is>
+      </c>
       <c r="J234" t="inlineStr"/>
       <c r="K234" t="inlineStr"/>
       <c r="L234" t="inlineStr"/>
@@ -13883,7 +14107,11 @@
       <c r="F235" t="inlineStr"/>
       <c r="G235" t="inlineStr"/>
       <c r="H235" t="inlineStr"/>
-      <c r="I235" t="inlineStr"/>
+      <c r="I235" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J235" t="inlineStr"/>
       <c r="K235" t="inlineStr"/>
       <c r="L235" t="inlineStr"/>
@@ -14219,7 +14447,7 @@
       <c r="H241" t="inlineStr"/>
       <c r="I241" t="inlineStr">
         <is>
-          <t>Black/African</t>
+          <t>White/European</t>
         </is>
       </c>
       <c r="J241" t="inlineStr"/>
@@ -14337,7 +14565,7 @@
       <c r="H243" t="inlineStr"/>
       <c r="I243" t="inlineStr">
         <is>
-          <t>White/European</t>
+          <t>Black/African</t>
         </is>
       </c>
       <c r="J243" t="inlineStr"/>
@@ -14394,7 +14622,11 @@
       <c r="F244" t="inlineStr"/>
       <c r="G244" t="inlineStr"/>
       <c r="H244" t="inlineStr"/>
-      <c r="I244" t="inlineStr"/>
+      <c r="I244" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J244" t="inlineStr"/>
       <c r="K244" t="inlineStr"/>
       <c r="L244" t="inlineStr"/>
@@ -14508,7 +14740,11 @@
       <c r="F246" t="inlineStr"/>
       <c r="G246" t="inlineStr"/>
       <c r="H246" t="inlineStr"/>
-      <c r="I246" t="inlineStr"/>
+      <c r="I246" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J246" t="inlineStr"/>
       <c r="K246" t="inlineStr"/>
       <c r="L246" t="inlineStr"/>
@@ -14575,7 +14811,11 @@
       <c r="F247" t="inlineStr"/>
       <c r="G247" t="inlineStr"/>
       <c r="H247" t="inlineStr"/>
-      <c r="I247" t="inlineStr"/>
+      <c r="I247" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J247" t="inlineStr"/>
       <c r="K247" t="inlineStr"/>
       <c r="L247" t="inlineStr"/>
@@ -15139,7 +15379,7 @@
       <c r="H257" t="inlineStr"/>
       <c r="I257" t="inlineStr">
         <is>
-          <t>Middle Eastern/Arab</t>
+          <t>Black/African</t>
         </is>
       </c>
       <c r="J257" t="inlineStr"/>
@@ -15196,7 +15436,11 @@
       <c r="F258" t="inlineStr"/>
       <c r="G258" t="inlineStr"/>
       <c r="H258" t="inlineStr"/>
-      <c r="I258" t="inlineStr"/>
+      <c r="I258" t="inlineStr">
+        <is>
+          <t>Mixed/Ambiguous</t>
+        </is>
+      </c>
       <c r="J258" t="inlineStr"/>
       <c r="K258" t="inlineStr"/>
       <c r="L258" t="inlineStr"/>
@@ -15322,7 +15566,11 @@
       <c r="F260" t="inlineStr"/>
       <c r="G260" t="inlineStr"/>
       <c r="H260" t="inlineStr"/>
-      <c r="I260" t="inlineStr"/>
+      <c r="I260" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J260" t="inlineStr"/>
       <c r="K260" t="inlineStr"/>
       <c r="L260" t="inlineStr"/>
@@ -15377,7 +15625,11 @@
       <c r="F261" t="inlineStr"/>
       <c r="G261" t="inlineStr"/>
       <c r="H261" t="inlineStr"/>
-      <c r="I261" t="inlineStr"/>
+      <c r="I261" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J261" t="inlineStr"/>
       <c r="K261" t="inlineStr"/>
       <c r="L261" t="inlineStr"/>
@@ -16057,7 +16309,11 @@
       <c r="F273" t="inlineStr"/>
       <c r="G273" t="inlineStr"/>
       <c r="H273" t="inlineStr"/>
-      <c r="I273" t="inlineStr"/>
+      <c r="I273" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J273" t="inlineStr"/>
       <c r="K273" t="inlineStr"/>
       <c r="L273" t="inlineStr"/>
@@ -16238,7 +16494,11 @@
       <c r="F276" t="inlineStr"/>
       <c r="G276" t="inlineStr"/>
       <c r="H276" t="inlineStr"/>
-      <c r="I276" t="inlineStr"/>
+      <c r="I276" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J276" t="inlineStr"/>
       <c r="K276" t="inlineStr"/>
       <c r="L276" t="inlineStr"/>
@@ -16427,7 +16687,11 @@
       <c r="F279" t="inlineStr"/>
       <c r="G279" t="inlineStr"/>
       <c r="H279" t="inlineStr"/>
-      <c r="I279" t="inlineStr"/>
+      <c r="I279" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J279" t="inlineStr"/>
       <c r="K279" t="inlineStr"/>
       <c r="L279" t="inlineStr"/>
@@ -16977,7 +17241,11 @@
       <c r="F289" t="inlineStr"/>
       <c r="G289" t="inlineStr"/>
       <c r="H289" t="inlineStr"/>
-      <c r="I289" t="inlineStr"/>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J289" t="inlineStr"/>
       <c r="K289" t="inlineStr"/>
       <c r="L289" t="inlineStr"/>
@@ -17087,7 +17355,11 @@
       <c r="F291" t="inlineStr"/>
       <c r="G291" t="inlineStr"/>
       <c r="H291" t="inlineStr"/>
-      <c r="I291" t="inlineStr"/>
+      <c r="I291" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J291" t="inlineStr"/>
       <c r="K291" t="inlineStr"/>
       <c r="L291" t="inlineStr"/>
@@ -17197,7 +17469,11 @@
       <c r="F293" t="inlineStr"/>
       <c r="G293" t="inlineStr"/>
       <c r="H293" t="inlineStr"/>
-      <c r="I293" t="inlineStr"/>
+      <c r="I293" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J293" t="inlineStr"/>
       <c r="K293" t="inlineStr"/>
       <c r="L293" t="inlineStr"/>
@@ -17307,7 +17583,11 @@
       <c r="F295" t="inlineStr"/>
       <c r="G295" t="inlineStr"/>
       <c r="H295" t="inlineStr"/>
-      <c r="I295" t="inlineStr"/>
+      <c r="I295" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J295" t="inlineStr"/>
       <c r="K295" t="inlineStr"/>
       <c r="L295" t="inlineStr"/>
@@ -17834,7 +18114,11 @@
       <c r="F304" t="inlineStr"/>
       <c r="G304" t="inlineStr"/>
       <c r="H304" t="inlineStr"/>
-      <c r="I304" t="inlineStr"/>
+      <c r="I304" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J304" t="inlineStr"/>
       <c r="K304" t="inlineStr"/>
       <c r="L304" t="inlineStr"/>
@@ -17889,7 +18173,11 @@
       <c r="F305" t="inlineStr"/>
       <c r="G305" t="inlineStr"/>
       <c r="H305" t="inlineStr"/>
-      <c r="I305" t="inlineStr"/>
+      <c r="I305" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J305" t="inlineStr"/>
       <c r="K305" t="inlineStr"/>
       <c r="L305" t="inlineStr"/>
@@ -18113,7 +18401,11 @@
       <c r="F309" t="inlineStr"/>
       <c r="G309" t="inlineStr"/>
       <c r="H309" t="inlineStr"/>
-      <c r="I309" t="inlineStr"/>
+      <c r="I309" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J309" t="inlineStr"/>
       <c r="K309" t="inlineStr"/>
       <c r="L309" t="inlineStr"/>
@@ -18282,7 +18574,11 @@
       <c r="F312" t="inlineStr"/>
       <c r="G312" t="inlineStr"/>
       <c r="H312" t="inlineStr"/>
-      <c r="I312" t="inlineStr"/>
+      <c r="I312" t="inlineStr">
+        <is>
+          <t>South Asian</t>
+        </is>
+      </c>
       <c r="J312" t="inlineStr"/>
       <c r="K312" t="inlineStr"/>
       <c r="L312" t="inlineStr"/>
@@ -18451,7 +18747,11 @@
       <c r="F315" t="inlineStr"/>
       <c r="G315" t="inlineStr"/>
       <c r="H315" t="inlineStr"/>
-      <c r="I315" t="inlineStr"/>
+      <c r="I315" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J315" t="inlineStr"/>
       <c r="K315" t="inlineStr"/>
       <c r="L315" t="inlineStr"/>
@@ -18620,7 +18920,11 @@
       <c r="F318" t="inlineStr"/>
       <c r="G318" t="inlineStr"/>
       <c r="H318" t="inlineStr"/>
-      <c r="I318" t="inlineStr"/>
+      <c r="I318" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J318" t="inlineStr"/>
       <c r="K318" t="inlineStr"/>
       <c r="L318" t="inlineStr"/>
@@ -19009,7 +19313,11 @@
       <c r="F325" t="inlineStr"/>
       <c r="G325" t="inlineStr"/>
       <c r="H325" t="inlineStr"/>
-      <c r="I325" t="inlineStr"/>
+      <c r="I325" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J325" t="inlineStr"/>
       <c r="K325" t="inlineStr"/>
       <c r="L325" t="inlineStr"/>
@@ -19066,7 +19374,7 @@
       <c r="H326" t="inlineStr"/>
       <c r="I326" t="inlineStr">
         <is>
-          <t>Hispanic/Latino</t>
+          <t>Middle Eastern/Arab</t>
         </is>
       </c>
       <c r="J326" t="inlineStr"/>
@@ -19241,7 +19549,11 @@
       <c r="F329" t="inlineStr"/>
       <c r="G329" t="inlineStr"/>
       <c r="H329" t="inlineStr"/>
-      <c r="I329" t="inlineStr"/>
+      <c r="I329" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J329" t="inlineStr"/>
       <c r="K329" t="inlineStr"/>
       <c r="L329" t="inlineStr"/>
@@ -19351,7 +19663,11 @@
       <c r="F331" t="inlineStr"/>
       <c r="G331" t="inlineStr"/>
       <c r="H331" t="inlineStr"/>
-      <c r="I331" t="inlineStr"/>
+      <c r="I331" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J331" t="inlineStr"/>
       <c r="K331" t="inlineStr"/>
       <c r="L331" t="inlineStr"/>
@@ -19465,7 +19781,11 @@
       <c r="F333" t="inlineStr"/>
       <c r="G333" t="inlineStr"/>
       <c r="H333" t="inlineStr"/>
-      <c r="I333" t="inlineStr"/>
+      <c r="I333" t="inlineStr">
+        <is>
+          <t>Mixed/Ambiguous</t>
+        </is>
+      </c>
       <c r="J333" t="inlineStr"/>
       <c r="K333" t="inlineStr"/>
       <c r="L333" t="inlineStr"/>
@@ -19575,7 +19895,11 @@
       <c r="F335" t="inlineStr"/>
       <c r="G335" t="inlineStr"/>
       <c r="H335" t="inlineStr"/>
-      <c r="I335" t="inlineStr"/>
+      <c r="I335" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J335" t="inlineStr"/>
       <c r="K335" t="inlineStr"/>
       <c r="L335" t="inlineStr"/>
@@ -19630,7 +19954,11 @@
       <c r="F336" t="inlineStr"/>
       <c r="G336" t="inlineStr"/>
       <c r="H336" t="inlineStr"/>
-      <c r="I336" t="inlineStr"/>
+      <c r="I336" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J336" t="inlineStr"/>
       <c r="K336" t="inlineStr"/>
       <c r="L336" t="inlineStr"/>
@@ -19795,7 +20123,11 @@
       <c r="F339" t="inlineStr"/>
       <c r="G339" t="inlineStr"/>
       <c r="H339" t="inlineStr"/>
-      <c r="I339" t="inlineStr"/>
+      <c r="I339" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J339" t="inlineStr"/>
       <c r="K339" t="inlineStr"/>
       <c r="L339" t="inlineStr"/>
@@ -19909,7 +20241,11 @@
       <c r="F341" t="inlineStr"/>
       <c r="G341" t="inlineStr"/>
       <c r="H341" t="inlineStr"/>
-      <c r="I341" t="inlineStr"/>
+      <c r="I341" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J341" t="inlineStr"/>
       <c r="K341" t="inlineStr"/>
       <c r="L341" t="inlineStr"/>
@@ -20033,7 +20369,7 @@
       <c r="H343" t="inlineStr"/>
       <c r="I343" t="inlineStr">
         <is>
-          <t>Middle Eastern/Arab</t>
+          <t>White/European</t>
         </is>
       </c>
       <c r="J343" t="inlineStr"/>
@@ -20265,7 +20601,7 @@
       <c r="H347" t="inlineStr"/>
       <c r="I347" t="inlineStr">
         <is>
-          <t>Black/African</t>
+          <t>Mixed/Ambiguous</t>
         </is>
       </c>
       <c r="J347" t="inlineStr"/>
@@ -20324,7 +20660,7 @@
       <c r="H348" t="inlineStr"/>
       <c r="I348" t="inlineStr">
         <is>
-          <t>Hispanic/Latino</t>
+          <t>White/European</t>
         </is>
       </c>
       <c r="J348" t="inlineStr"/>
@@ -20605,7 +20941,11 @@
       <c r="F353" t="inlineStr"/>
       <c r="G353" t="inlineStr"/>
       <c r="H353" t="inlineStr"/>
-      <c r="I353" t="inlineStr"/>
+      <c r="I353" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J353" t="inlineStr"/>
       <c r="K353" t="inlineStr"/>
       <c r="L353" t="inlineStr"/>
@@ -20719,7 +21059,11 @@
       <c r="F355" t="inlineStr"/>
       <c r="G355" t="inlineStr"/>
       <c r="H355" t="inlineStr"/>
-      <c r="I355" t="inlineStr"/>
+      <c r="I355" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J355" t="inlineStr"/>
       <c r="K355" t="inlineStr"/>
       <c r="L355" t="inlineStr"/>
@@ -20829,7 +21173,11 @@
       <c r="F357" t="inlineStr"/>
       <c r="G357" t="inlineStr"/>
       <c r="H357" t="inlineStr"/>
-      <c r="I357" t="inlineStr"/>
+      <c r="I357" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J357" t="inlineStr"/>
       <c r="K357" t="inlineStr"/>
       <c r="L357" t="inlineStr"/>
@@ -20939,7 +21287,11 @@
       <c r="F359" t="inlineStr"/>
       <c r="G359" t="inlineStr"/>
       <c r="H359" t="inlineStr"/>
-      <c r="I359" t="inlineStr"/>
+      <c r="I359" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J359" t="inlineStr"/>
       <c r="K359" t="inlineStr"/>
       <c r="L359" t="inlineStr"/>
@@ -21049,7 +21401,11 @@
       <c r="F361" t="inlineStr"/>
       <c r="G361" t="inlineStr"/>
       <c r="H361" t="inlineStr"/>
-      <c r="I361" t="inlineStr"/>
+      <c r="I361" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J361" t="inlineStr"/>
       <c r="K361" t="inlineStr"/>
       <c r="L361" t="inlineStr"/>
@@ -21175,7 +21531,11 @@
       <c r="F363" t="inlineStr"/>
       <c r="G363" t="inlineStr"/>
       <c r="H363" t="inlineStr"/>
-      <c r="I363" t="inlineStr"/>
+      <c r="I363" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J363" t="inlineStr"/>
       <c r="K363" t="inlineStr"/>
       <c r="L363" t="inlineStr"/>
@@ -21285,7 +21645,11 @@
       <c r="F365" t="inlineStr"/>
       <c r="G365" t="inlineStr"/>
       <c r="H365" t="inlineStr"/>
-      <c r="I365" t="inlineStr"/>
+      <c r="I365" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J365" t="inlineStr"/>
       <c r="K365" t="inlineStr"/>
       <c r="L365" t="inlineStr"/>
@@ -21340,7 +21704,11 @@
       <c r="F366" t="inlineStr"/>
       <c r="G366" t="inlineStr"/>
       <c r="H366" t="inlineStr"/>
-      <c r="I366" t="inlineStr"/>
+      <c r="I366" t="inlineStr">
+        <is>
+          <t>South Asian</t>
+        </is>
+      </c>
       <c r="J366" t="inlineStr"/>
       <c r="K366" t="inlineStr"/>
       <c r="L366" t="inlineStr"/>
@@ -21450,7 +21818,11 @@
       <c r="F368" t="inlineStr"/>
       <c r="G368" t="inlineStr"/>
       <c r="H368" t="inlineStr"/>
-      <c r="I368" t="inlineStr"/>
+      <c r="I368" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J368" t="inlineStr"/>
       <c r="K368" t="inlineStr"/>
       <c r="L368" t="inlineStr"/>
@@ -21560,7 +21932,11 @@
       <c r="F370" t="inlineStr"/>
       <c r="G370" t="inlineStr"/>
       <c r="H370" t="inlineStr"/>
-      <c r="I370" t="inlineStr"/>
+      <c r="I370" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J370" t="inlineStr"/>
       <c r="K370" t="inlineStr"/>
       <c r="L370" t="inlineStr"/>
@@ -21906,7 +22282,11 @@
       <c r="F376" t="inlineStr"/>
       <c r="G376" t="inlineStr"/>
       <c r="H376" t="inlineStr"/>
-      <c r="I376" t="inlineStr"/>
+      <c r="I376" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J376" t="inlineStr"/>
       <c r="K376" t="inlineStr"/>
       <c r="L376" t="inlineStr"/>
@@ -22413,7 +22793,11 @@
       <c r="F385" t="inlineStr"/>
       <c r="G385" t="inlineStr"/>
       <c r="H385" t="inlineStr"/>
-      <c r="I385" t="inlineStr"/>
+      <c r="I385" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J385" t="inlineStr"/>
       <c r="K385" t="inlineStr"/>
       <c r="L385" t="inlineStr"/>
@@ -22523,7 +22907,11 @@
       <c r="F387" t="inlineStr"/>
       <c r="G387" t="inlineStr"/>
       <c r="H387" t="inlineStr"/>
-      <c r="I387" t="inlineStr"/>
+      <c r="I387" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J387" t="inlineStr"/>
       <c r="K387" t="inlineStr"/>
       <c r="L387" t="inlineStr"/>
@@ -22578,7 +22966,11 @@
       <c r="F388" t="inlineStr"/>
       <c r="G388" t="inlineStr"/>
       <c r="H388" t="inlineStr"/>
-      <c r="I388" t="inlineStr"/>
+      <c r="I388" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J388" t="inlineStr"/>
       <c r="K388" t="inlineStr"/>
       <c r="L388" t="inlineStr"/>
@@ -22700,7 +23092,11 @@
       <c r="F390" t="inlineStr"/>
       <c r="G390" t="inlineStr"/>
       <c r="H390" t="inlineStr"/>
-      <c r="I390" t="inlineStr"/>
+      <c r="I390" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J390" t="inlineStr"/>
       <c r="K390" t="inlineStr"/>
       <c r="L390" t="inlineStr"/>
@@ -22755,7 +23151,11 @@
       <c r="F391" t="inlineStr"/>
       <c r="G391" t="inlineStr"/>
       <c r="H391" t="inlineStr"/>
-      <c r="I391" t="inlineStr"/>
+      <c r="I391" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J391" t="inlineStr"/>
       <c r="K391" t="inlineStr"/>
       <c r="L391" t="inlineStr"/>
@@ -23364,7 +23764,11 @@
       <c r="F402" t="inlineStr"/>
       <c r="G402" t="inlineStr"/>
       <c r="H402" t="inlineStr"/>
-      <c r="I402" t="inlineStr"/>
+      <c r="I402" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J402" t="inlineStr"/>
       <c r="K402" t="inlineStr"/>
       <c r="L402" t="inlineStr"/>
@@ -23486,7 +23890,11 @@
       <c r="F404" t="inlineStr"/>
       <c r="G404" t="inlineStr"/>
       <c r="H404" t="inlineStr"/>
-      <c r="I404" t="inlineStr"/>
+      <c r="I404" t="inlineStr">
+        <is>
+          <t>Middle Eastern/Arab</t>
+        </is>
+      </c>
       <c r="J404" t="inlineStr"/>
       <c r="K404" t="inlineStr"/>
       <c r="L404" t="inlineStr"/>
@@ -23541,7 +23949,11 @@
       <c r="F405" t="inlineStr"/>
       <c r="G405" t="inlineStr"/>
       <c r="H405" t="inlineStr"/>
-      <c r="I405" t="inlineStr"/>
+      <c r="I405" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J405" t="inlineStr"/>
       <c r="K405" t="inlineStr"/>
       <c r="L405" t="inlineStr"/>
@@ -23596,7 +24008,11 @@
       <c r="F406" t="inlineStr"/>
       <c r="G406" t="inlineStr"/>
       <c r="H406" t="inlineStr"/>
-      <c r="I406" t="inlineStr"/>
+      <c r="I406" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J406" t="inlineStr"/>
       <c r="K406" t="inlineStr"/>
       <c r="L406" t="inlineStr"/>
@@ -23663,7 +24079,11 @@
       <c r="F407" t="inlineStr"/>
       <c r="G407" t="inlineStr"/>
       <c r="H407" t="inlineStr"/>
-      <c r="I407" t="inlineStr"/>
+      <c r="I407" t="inlineStr">
+        <is>
+          <t>Hispanic/Latino</t>
+        </is>
+      </c>
       <c r="J407" t="inlineStr"/>
       <c r="K407" t="inlineStr"/>
       <c r="L407" t="inlineStr"/>
@@ -23883,7 +24303,11 @@
       <c r="F411" t="inlineStr"/>
       <c r="G411" t="inlineStr"/>
       <c r="H411" t="inlineStr"/>
-      <c r="I411" t="inlineStr"/>
+      <c r="I411" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J411" t="inlineStr"/>
       <c r="K411" t="inlineStr"/>
       <c r="L411" t="inlineStr"/>
@@ -23993,7 +24417,11 @@
       <c r="F413" t="inlineStr"/>
       <c r="G413" t="inlineStr"/>
       <c r="H413" t="inlineStr"/>
-      <c r="I413" t="inlineStr"/>
+      <c r="I413" t="inlineStr">
+        <is>
+          <t>South Asian</t>
+        </is>
+      </c>
       <c r="J413" t="inlineStr"/>
       <c r="K413" t="inlineStr"/>
       <c r="L413" t="inlineStr"/>
@@ -24217,7 +24645,11 @@
       <c r="F417" t="inlineStr"/>
       <c r="G417" t="inlineStr"/>
       <c r="H417" t="inlineStr"/>
-      <c r="I417" t="inlineStr"/>
+      <c r="I417" t="inlineStr">
+        <is>
+          <t>South Asian</t>
+        </is>
+      </c>
       <c r="J417" t="inlineStr"/>
       <c r="K417" t="inlineStr"/>
       <c r="L417" t="inlineStr"/>
@@ -24272,7 +24704,11 @@
       <c r="F418" t="inlineStr"/>
       <c r="G418" t="inlineStr"/>
       <c r="H418" t="inlineStr"/>
-      <c r="I418" t="inlineStr"/>
+      <c r="I418" t="inlineStr">
+        <is>
+          <t>South Asian</t>
+        </is>
+      </c>
       <c r="J418" t="inlineStr"/>
       <c r="K418" t="inlineStr"/>
       <c r="L418" t="inlineStr"/>
@@ -24732,7 +25168,11 @@
       <c r="F426" t="inlineStr"/>
       <c r="G426" t="inlineStr"/>
       <c r="H426" t="inlineStr"/>
-      <c r="I426" t="inlineStr"/>
+      <c r="I426" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J426" t="inlineStr"/>
       <c r="K426" t="inlineStr"/>
       <c r="L426" t="inlineStr"/>
@@ -24976,7 +25416,11 @@
           <t>25-34</t>
         </is>
       </c>
-      <c r="I430" t="inlineStr"/>
+      <c r="I430" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J430" t="inlineStr">
         <is>
           <t>5.85</t>
@@ -25216,7 +25660,11 @@
       <c r="F434" t="inlineStr"/>
       <c r="G434" t="inlineStr"/>
       <c r="H434" t="inlineStr"/>
-      <c r="I434" t="inlineStr"/>
+      <c r="I434" t="inlineStr">
+        <is>
+          <t>South Asian</t>
+        </is>
+      </c>
       <c r="J434" t="inlineStr"/>
       <c r="K434" t="inlineStr"/>
       <c r="L434" t="inlineStr"/>
@@ -25332,7 +25780,7 @@
       <c r="H436" t="inlineStr"/>
       <c r="I436" t="inlineStr">
         <is>
-          <t>Middle Eastern/Arab</t>
+          <t>Mixed/Ambiguous</t>
         </is>
       </c>
       <c r="J436" t="inlineStr"/>
@@ -25499,7 +25947,11 @@
       <c r="F439" t="inlineStr"/>
       <c r="G439" t="inlineStr"/>
       <c r="H439" t="inlineStr"/>
-      <c r="I439" t="inlineStr"/>
+      <c r="I439" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J439" t="inlineStr"/>
       <c r="K439" t="inlineStr"/>
       <c r="L439" t="inlineStr"/>
@@ -25611,7 +26063,7 @@
       <c r="H441" t="inlineStr"/>
       <c r="I441" t="inlineStr">
         <is>
-          <t>Black/African</t>
+          <t>Mixed/Ambiguous</t>
         </is>
       </c>
       <c r="J441" t="inlineStr"/>
@@ -25668,7 +26120,11 @@
       <c r="F442" t="inlineStr"/>
       <c r="G442" t="inlineStr"/>
       <c r="H442" t="inlineStr"/>
-      <c r="I442" t="inlineStr"/>
+      <c r="I442" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J442" t="inlineStr"/>
       <c r="K442" t="inlineStr"/>
       <c r="L442" t="inlineStr"/>
@@ -26242,7 +26698,11 @@
       <c r="F452" t="inlineStr"/>
       <c r="G452" t="inlineStr"/>
       <c r="H452" t="inlineStr"/>
-      <c r="I452" t="inlineStr"/>
+      <c r="I452" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J452" t="inlineStr"/>
       <c r="K452" t="inlineStr"/>
       <c r="L452" t="inlineStr"/>
@@ -26297,7 +26757,11 @@
       <c r="F453" t="inlineStr"/>
       <c r="G453" t="inlineStr"/>
       <c r="H453" t="inlineStr"/>
-      <c r="I453" t="inlineStr"/>
+      <c r="I453" t="inlineStr">
+        <is>
+          <t>Middle Eastern/Arab</t>
+        </is>
+      </c>
       <c r="J453" t="inlineStr"/>
       <c r="K453" t="inlineStr"/>
       <c r="L453" t="inlineStr"/>
@@ -26407,7 +26871,11 @@
       <c r="F455" t="inlineStr"/>
       <c r="G455" t="inlineStr"/>
       <c r="H455" t="inlineStr"/>
-      <c r="I455" t="inlineStr"/>
+      <c r="I455" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J455" t="inlineStr"/>
       <c r="K455" t="inlineStr"/>
       <c r="L455" t="inlineStr"/>
@@ -26753,7 +27221,11 @@
       <c r="F461" t="inlineStr"/>
       <c r="G461" t="inlineStr"/>
       <c r="H461" t="inlineStr"/>
-      <c r="I461" t="inlineStr"/>
+      <c r="I461" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J461" t="inlineStr"/>
       <c r="K461" t="inlineStr"/>
       <c r="L461" t="inlineStr"/>
@@ -27225,7 +27697,11 @@
       <c r="F469" t="inlineStr"/>
       <c r="G469" t="inlineStr"/>
       <c r="H469" t="inlineStr"/>
-      <c r="I469" t="inlineStr"/>
+      <c r="I469" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J469" t="inlineStr"/>
       <c r="K469" t="inlineStr"/>
       <c r="L469" t="inlineStr"/>
@@ -27736,7 +28212,11 @@
       <c r="F478" t="inlineStr"/>
       <c r="G478" t="inlineStr"/>
       <c r="H478" t="inlineStr"/>
-      <c r="I478" t="inlineStr"/>
+      <c r="I478" t="inlineStr">
+        <is>
+          <t>Mixed/Ambiguous</t>
+        </is>
+      </c>
       <c r="J478" t="inlineStr"/>
       <c r="K478" t="inlineStr"/>
       <c r="L478" t="inlineStr"/>
@@ -27791,7 +28271,11 @@
       <c r="F479" t="inlineStr"/>
       <c r="G479" t="inlineStr"/>
       <c r="H479" t="inlineStr"/>
-      <c r="I479" t="inlineStr"/>
+      <c r="I479" t="inlineStr">
+        <is>
+          <t>Hispanic/Latino</t>
+        </is>
+      </c>
       <c r="J479" t="inlineStr"/>
       <c r="K479" t="inlineStr"/>
       <c r="L479" t="inlineStr"/>
@@ -27917,7 +28401,11 @@
       <c r="F481" t="inlineStr"/>
       <c r="G481" t="inlineStr"/>
       <c r="H481" t="inlineStr"/>
-      <c r="I481" t="inlineStr"/>
+      <c r="I481" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J481" t="inlineStr"/>
       <c r="K481" t="inlineStr"/>
       <c r="L481" t="inlineStr"/>
@@ -28204,7 +28692,11 @@
       <c r="F486" t="inlineStr"/>
       <c r="G486" t="inlineStr"/>
       <c r="H486" t="inlineStr"/>
-      <c r="I486" t="inlineStr"/>
+      <c r="I486" t="inlineStr">
+        <is>
+          <t>South Asian</t>
+        </is>
+      </c>
       <c r="J486" t="inlineStr"/>
       <c r="K486" t="inlineStr"/>
       <c r="L486" t="inlineStr"/>
@@ -28259,7 +28751,11 @@
       <c r="F487" t="inlineStr"/>
       <c r="G487" t="inlineStr"/>
       <c r="H487" t="inlineStr"/>
-      <c r="I487" t="inlineStr"/>
+      <c r="I487" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J487" t="inlineStr"/>
       <c r="K487" t="inlineStr"/>
       <c r="L487" t="inlineStr"/>
@@ -29289,7 +29785,11 @@
       <c r="F505" t="inlineStr"/>
       <c r="G505" t="inlineStr"/>
       <c r="H505" t="inlineStr"/>
-      <c r="I505" t="inlineStr"/>
+      <c r="I505" t="inlineStr">
+        <is>
+          <t>Middle Eastern/Arab</t>
+        </is>
+      </c>
       <c r="J505" t="inlineStr"/>
       <c r="K505" t="inlineStr"/>
       <c r="L505" t="inlineStr"/>
@@ -29454,7 +29954,11 @@
       <c r="F508" t="inlineStr"/>
       <c r="G508" t="inlineStr"/>
       <c r="H508" t="inlineStr"/>
-      <c r="I508" t="inlineStr"/>
+      <c r="I508" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J508" t="inlineStr"/>
       <c r="K508" t="inlineStr"/>
       <c r="L508" t="inlineStr"/>
@@ -29564,7 +30068,11 @@
       <c r="F510" t="inlineStr"/>
       <c r="G510" t="inlineStr"/>
       <c r="H510" t="inlineStr"/>
-      <c r="I510" t="inlineStr"/>
+      <c r="I510" t="inlineStr">
+        <is>
+          <t>Middle Eastern/Arab</t>
+        </is>
+      </c>
       <c r="J510" t="inlineStr"/>
       <c r="K510" t="inlineStr"/>
       <c r="L510" t="inlineStr"/>
@@ -29847,7 +30355,11 @@
       <c r="F515" t="inlineStr"/>
       <c r="G515" t="inlineStr"/>
       <c r="H515" t="inlineStr"/>
-      <c r="I515" t="inlineStr"/>
+      <c r="I515" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J515" t="inlineStr"/>
       <c r="K515" t="inlineStr"/>
       <c r="L515" t="inlineStr"/>
@@ -29961,7 +30473,11 @@
       <c r="F517" t="inlineStr"/>
       <c r="G517" t="inlineStr"/>
       <c r="H517" t="inlineStr"/>
-      <c r="I517" t="inlineStr"/>
+      <c r="I517" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J517" t="inlineStr"/>
       <c r="K517" t="inlineStr"/>
       <c r="L517" t="inlineStr"/>
@@ -30468,7 +30984,11 @@
       <c r="F526" t="inlineStr"/>
       <c r="G526" t="inlineStr"/>
       <c r="H526" t="inlineStr"/>
-      <c r="I526" t="inlineStr"/>
+      <c r="I526" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J526" t="inlineStr"/>
       <c r="K526" t="inlineStr"/>
       <c r="L526" t="inlineStr"/>
@@ -31148,7 +31668,11 @@
       <c r="F538" t="inlineStr"/>
       <c r="G538" t="inlineStr"/>
       <c r="H538" t="inlineStr"/>
-      <c r="I538" t="inlineStr"/>
+      <c r="I538" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J538" t="inlineStr"/>
       <c r="K538" t="inlineStr"/>
       <c r="L538" t="inlineStr"/>
@@ -31203,7 +31727,11 @@
       <c r="F539" t="inlineStr"/>
       <c r="G539" t="inlineStr"/>
       <c r="H539" t="inlineStr"/>
-      <c r="I539" t="inlineStr"/>
+      <c r="I539" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J539" t="inlineStr"/>
       <c r="K539" t="inlineStr"/>
       <c r="L539" t="inlineStr"/>
@@ -31258,7 +31786,11 @@
       <c r="F540" t="inlineStr"/>
       <c r="G540" t="inlineStr"/>
       <c r="H540" t="inlineStr"/>
-      <c r="I540" t="inlineStr"/>
+      <c r="I540" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J540" t="inlineStr"/>
       <c r="K540" t="inlineStr"/>
       <c r="L540" t="inlineStr"/>
@@ -31368,7 +31900,11 @@
       <c r="F542" t="inlineStr"/>
       <c r="G542" t="inlineStr"/>
       <c r="H542" t="inlineStr"/>
-      <c r="I542" t="inlineStr"/>
+      <c r="I542" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J542" t="inlineStr"/>
       <c r="K542" t="inlineStr"/>
       <c r="L542" t="inlineStr"/>
@@ -31478,7 +32014,11 @@
       <c r="F544" t="inlineStr"/>
       <c r="G544" t="inlineStr"/>
       <c r="H544" t="inlineStr"/>
-      <c r="I544" t="inlineStr"/>
+      <c r="I544" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J544" t="inlineStr"/>
       <c r="K544" t="inlineStr"/>
       <c r="L544" t="inlineStr"/>
@@ -31653,7 +32193,7 @@
       <c r="H547" t="inlineStr"/>
       <c r="I547" t="inlineStr">
         <is>
-          <t>Black/African</t>
+          <t>White/European</t>
         </is>
       </c>
       <c r="J547" t="inlineStr"/>
@@ -32174,7 +32714,11 @@
       <c r="F556" t="inlineStr"/>
       <c r="G556" t="inlineStr"/>
       <c r="H556" t="inlineStr"/>
-      <c r="I556" t="inlineStr"/>
+      <c r="I556" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J556" t="inlineStr"/>
       <c r="K556" t="inlineStr"/>
       <c r="L556" t="inlineStr"/>
@@ -32457,7 +33001,11 @@
       <c r="F561" t="inlineStr"/>
       <c r="G561" t="inlineStr"/>
       <c r="H561" t="inlineStr"/>
-      <c r="I561" t="inlineStr"/>
+      <c r="I561" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J561" t="inlineStr"/>
       <c r="K561" t="inlineStr"/>
       <c r="L561" t="inlineStr"/>
@@ -32681,7 +33229,11 @@
       <c r="F565" t="inlineStr"/>
       <c r="G565" t="inlineStr"/>
       <c r="H565" t="inlineStr"/>
-      <c r="I565" t="inlineStr"/>
+      <c r="I565" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J565" t="inlineStr"/>
       <c r="K565" t="inlineStr"/>
       <c r="L565" t="inlineStr"/>
@@ -32901,7 +33453,11 @@
       <c r="F569" t="inlineStr"/>
       <c r="G569" t="inlineStr"/>
       <c r="H569" t="inlineStr"/>
-      <c r="I569" t="inlineStr"/>
+      <c r="I569" t="inlineStr">
+        <is>
+          <t>South Asian</t>
+        </is>
+      </c>
       <c r="J569" t="inlineStr"/>
       <c r="K569" t="inlineStr"/>
       <c r="L569" t="inlineStr"/>
@@ -32956,7 +33512,11 @@
       <c r="F570" t="inlineStr"/>
       <c r="G570" t="inlineStr"/>
       <c r="H570" t="inlineStr"/>
-      <c r="I570" t="inlineStr"/>
+      <c r="I570" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J570" t="inlineStr"/>
       <c r="K570" t="inlineStr"/>
       <c r="L570" t="inlineStr"/>
@@ -33408,7 +33968,11 @@
       <c r="F578" t="inlineStr"/>
       <c r="G578" t="inlineStr"/>
       <c r="H578" t="inlineStr"/>
-      <c r="I578" t="inlineStr"/>
+      <c r="I578" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J578" t="inlineStr"/>
       <c r="K578" t="inlineStr"/>
       <c r="L578" t="inlineStr"/>
@@ -33852,7 +34416,11 @@
       <c r="F586" t="inlineStr"/>
       <c r="G586" t="inlineStr"/>
       <c r="H586" t="inlineStr"/>
-      <c r="I586" t="inlineStr"/>
+      <c r="I586" t="inlineStr">
+        <is>
+          <t>South Asian</t>
+        </is>
+      </c>
       <c r="J586" t="inlineStr"/>
       <c r="K586" t="inlineStr"/>
       <c r="L586" t="inlineStr"/>
@@ -34019,7 +34587,7 @@
       <c r="H589" t="inlineStr"/>
       <c r="I589" t="inlineStr">
         <is>
-          <t>Middle Eastern/Arab</t>
+          <t>South Asian</t>
         </is>
       </c>
       <c r="J589" t="inlineStr"/>
@@ -34245,7 +34813,11 @@
       <c r="F593" t="inlineStr"/>
       <c r="G593" t="inlineStr"/>
       <c r="H593" t="inlineStr"/>
-      <c r="I593" t="inlineStr"/>
+      <c r="I593" t="inlineStr">
+        <is>
+          <t>South Asian</t>
+        </is>
+      </c>
       <c r="J593" t="inlineStr"/>
       <c r="K593" t="inlineStr"/>
       <c r="L593" t="inlineStr"/>
@@ -34422,7 +34994,11 @@
       <c r="F596" t="inlineStr"/>
       <c r="G596" t="inlineStr"/>
       <c r="H596" t="inlineStr"/>
-      <c r="I596" t="inlineStr"/>
+      <c r="I596" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J596" t="inlineStr"/>
       <c r="K596" t="inlineStr"/>
       <c r="L596" t="inlineStr"/>
@@ -34532,7 +35108,11 @@
       <c r="F598" t="inlineStr"/>
       <c r="G598" t="inlineStr"/>
       <c r="H598" t="inlineStr"/>
-      <c r="I598" t="inlineStr"/>
+      <c r="I598" t="inlineStr">
+        <is>
+          <t>South Asian</t>
+        </is>
+      </c>
       <c r="J598" t="inlineStr"/>
       <c r="K598" t="inlineStr"/>
       <c r="L598" t="inlineStr"/>
@@ -34752,7 +35332,11 @@
       <c r="F602" t="inlineStr"/>
       <c r="G602" t="inlineStr"/>
       <c r="H602" t="inlineStr"/>
-      <c r="I602" t="inlineStr"/>
+      <c r="I602" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J602" t="inlineStr"/>
       <c r="K602" t="inlineStr"/>
       <c r="L602" t="inlineStr"/>
@@ -34929,7 +35513,11 @@
       <c r="F605" t="inlineStr"/>
       <c r="G605" t="inlineStr"/>
       <c r="H605" t="inlineStr"/>
-      <c r="I605" t="inlineStr"/>
+      <c r="I605" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J605" t="inlineStr"/>
       <c r="K605" t="inlineStr"/>
       <c r="L605" t="inlineStr"/>
@@ -34984,7 +35572,11 @@
       <c r="F606" t="inlineStr"/>
       <c r="G606" t="inlineStr"/>
       <c r="H606" t="inlineStr"/>
-      <c r="I606" t="inlineStr"/>
+      <c r="I606" t="inlineStr">
+        <is>
+          <t>South Asian</t>
+        </is>
+      </c>
       <c r="J606" t="inlineStr"/>
       <c r="K606" t="inlineStr"/>
       <c r="L606" t="inlineStr"/>
@@ -35263,7 +35855,11 @@
       <c r="F611" t="inlineStr"/>
       <c r="G611" t="inlineStr"/>
       <c r="H611" t="inlineStr"/>
-      <c r="I611" t="inlineStr"/>
+      <c r="I611" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J611" t="inlineStr"/>
       <c r="K611" t="inlineStr"/>
       <c r="L611" t="inlineStr"/>
@@ -35660,7 +36256,11 @@
       <c r="F618" t="inlineStr"/>
       <c r="G618" t="inlineStr"/>
       <c r="H618" t="inlineStr"/>
-      <c r="I618" t="inlineStr"/>
+      <c r="I618" t="inlineStr">
+        <is>
+          <t>South Asian</t>
+        </is>
+      </c>
       <c r="J618" t="inlineStr"/>
       <c r="K618" t="inlineStr"/>
       <c r="L618" t="inlineStr"/>
@@ -35939,7 +36539,11 @@
       <c r="F623" t="inlineStr"/>
       <c r="G623" t="inlineStr"/>
       <c r="H623" t="inlineStr"/>
-      <c r="I623" t="inlineStr"/>
+      <c r="I623" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J623" t="inlineStr"/>
       <c r="K623" t="inlineStr"/>
       <c r="L623" t="inlineStr"/>
@@ -36049,7 +36653,11 @@
       <c r="F625" t="inlineStr"/>
       <c r="G625" t="inlineStr"/>
       <c r="H625" t="inlineStr"/>
-      <c r="I625" t="inlineStr"/>
+      <c r="I625" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J625" t="inlineStr"/>
       <c r="K625" t="inlineStr"/>
       <c r="L625" t="inlineStr"/>
@@ -36344,7 +36952,11 @@
       <c r="F630" t="inlineStr"/>
       <c r="G630" t="inlineStr"/>
       <c r="H630" t="inlineStr"/>
-      <c r="I630" t="inlineStr"/>
+      <c r="I630" t="inlineStr">
+        <is>
+          <t>Mixed/Ambiguous</t>
+        </is>
+      </c>
       <c r="J630" t="inlineStr"/>
       <c r="K630" t="inlineStr"/>
       <c r="L630" t="inlineStr"/>
@@ -36741,7 +37353,11 @@
       <c r="F637" t="inlineStr"/>
       <c r="G637" t="inlineStr"/>
       <c r="H637" t="inlineStr"/>
-      <c r="I637" t="inlineStr"/>
+      <c r="I637" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J637" t="inlineStr"/>
       <c r="K637" t="inlineStr"/>
       <c r="L637" t="inlineStr"/>
@@ -36851,7 +37467,11 @@
       <c r="F639" t="inlineStr"/>
       <c r="G639" t="inlineStr"/>
       <c r="H639" t="inlineStr"/>
-      <c r="I639" t="inlineStr"/>
+      <c r="I639" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J639" t="inlineStr"/>
       <c r="K639" t="inlineStr"/>
       <c r="L639" t="inlineStr"/>
@@ -37079,7 +37699,11 @@
       <c r="F643" t="inlineStr"/>
       <c r="G643" t="inlineStr"/>
       <c r="H643" t="inlineStr"/>
-      <c r="I643" t="inlineStr"/>
+      <c r="I643" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J643" t="inlineStr"/>
       <c r="K643" t="inlineStr"/>
       <c r="L643" t="inlineStr"/>
@@ -37136,7 +37760,7 @@
       <c r="H644" t="inlineStr"/>
       <c r="I644" t="inlineStr">
         <is>
-          <t>White/European</t>
+          <t>South Asian</t>
         </is>
       </c>
       <c r="J644" t="inlineStr"/>
@@ -37250,7 +37874,7 @@
       <c r="H646" t="inlineStr"/>
       <c r="I646" t="inlineStr">
         <is>
-          <t>Black/African</t>
+          <t>South Asian</t>
         </is>
       </c>
       <c r="J646" t="inlineStr"/>
@@ -37362,7 +37986,11 @@
       <c r="F648" t="inlineStr"/>
       <c r="G648" t="inlineStr"/>
       <c r="H648" t="inlineStr"/>
-      <c r="I648" t="inlineStr"/>
+      <c r="I648" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J648" t="inlineStr"/>
       <c r="K648" t="inlineStr"/>
       <c r="L648" t="inlineStr"/>
@@ -37527,7 +38155,11 @@
       <c r="F651" t="inlineStr"/>
       <c r="G651" t="inlineStr"/>
       <c r="H651" t="inlineStr"/>
-      <c r="I651" t="inlineStr"/>
+      <c r="I651" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J651" t="inlineStr"/>
       <c r="K651" t="inlineStr"/>
       <c r="L651" t="inlineStr"/>
@@ -37641,7 +38273,11 @@
       <c r="F653" t="inlineStr"/>
       <c r="G653" t="inlineStr"/>
       <c r="H653" t="inlineStr"/>
-      <c r="I653" t="inlineStr"/>
+      <c r="I653" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J653" t="inlineStr"/>
       <c r="K653" t="inlineStr"/>
       <c r="L653" t="inlineStr"/>
@@ -37810,7 +38446,11 @@
       <c r="F656" t="inlineStr"/>
       <c r="G656" t="inlineStr"/>
       <c r="H656" t="inlineStr"/>
-      <c r="I656" t="inlineStr"/>
+      <c r="I656" t="inlineStr">
+        <is>
+          <t>Mixed/Ambiguous</t>
+        </is>
+      </c>
       <c r="J656" t="inlineStr"/>
       <c r="K656" t="inlineStr"/>
       <c r="L656" t="inlineStr"/>
@@ -37979,7 +38619,11 @@
       <c r="F659" t="inlineStr"/>
       <c r="G659" t="inlineStr"/>
       <c r="H659" t="inlineStr"/>
-      <c r="I659" t="inlineStr"/>
+      <c r="I659" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J659" t="inlineStr"/>
       <c r="K659" t="inlineStr"/>
       <c r="L659" t="inlineStr"/>
@@ -38374,7 +39018,7 @@
       <c r="H666" t="inlineStr"/>
       <c r="I666" t="inlineStr">
         <is>
-          <t>East/SE Asian</t>
+          <t>Black/African</t>
         </is>
       </c>
       <c r="J666" t="inlineStr"/>
@@ -38608,7 +39252,11 @@
       <c r="F670" t="inlineStr"/>
       <c r="G670" t="inlineStr"/>
       <c r="H670" t="inlineStr"/>
-      <c r="I670" t="inlineStr"/>
+      <c r="I670" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J670" t="inlineStr"/>
       <c r="K670" t="inlineStr"/>
       <c r="L670" t="inlineStr"/>
@@ -38844,7 +39492,11 @@
       <c r="F674" t="inlineStr"/>
       <c r="G674" t="inlineStr"/>
       <c r="H674" t="inlineStr"/>
-      <c r="I674" t="inlineStr"/>
+      <c r="I674" t="inlineStr">
+        <is>
+          <t>Mixed/Ambiguous</t>
+        </is>
+      </c>
       <c r="J674" t="inlineStr"/>
       <c r="K674" t="inlineStr"/>
       <c r="L674" t="inlineStr"/>
@@ -39068,7 +39720,11 @@
       <c r="F678" t="inlineStr"/>
       <c r="G678" t="inlineStr"/>
       <c r="H678" t="inlineStr"/>
-      <c r="I678" t="inlineStr"/>
+      <c r="I678" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J678" t="inlineStr"/>
       <c r="K678" t="inlineStr"/>
       <c r="L678" t="inlineStr"/>
@@ -39178,7 +39834,11 @@
       <c r="F680" t="inlineStr"/>
       <c r="G680" t="inlineStr"/>
       <c r="H680" t="inlineStr"/>
-      <c r="I680" t="inlineStr"/>
+      <c r="I680" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J680" t="inlineStr"/>
       <c r="K680" t="inlineStr"/>
       <c r="L680" t="inlineStr"/>
@@ -39414,7 +40074,11 @@
       <c r="F684" t="inlineStr"/>
       <c r="G684" t="inlineStr"/>
       <c r="H684" t="inlineStr"/>
-      <c r="I684" t="inlineStr"/>
+      <c r="I684" t="inlineStr">
+        <is>
+          <t>Mixed/Ambiguous</t>
+        </is>
+      </c>
       <c r="J684" t="inlineStr"/>
       <c r="K684" t="inlineStr"/>
       <c r="L684" t="inlineStr"/>
@@ -39481,7 +40145,11 @@
       <c r="F685" t="inlineStr"/>
       <c r="G685" t="inlineStr"/>
       <c r="H685" t="inlineStr"/>
-      <c r="I685" t="inlineStr"/>
+      <c r="I685" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J685" t="inlineStr"/>
       <c r="K685" t="inlineStr"/>
       <c r="L685" t="inlineStr"/>
@@ -39536,7 +40204,11 @@
       <c r="F686" t="inlineStr"/>
       <c r="G686" t="inlineStr"/>
       <c r="H686" t="inlineStr"/>
-      <c r="I686" t="inlineStr"/>
+      <c r="I686" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J686" t="inlineStr"/>
       <c r="K686" t="inlineStr"/>
       <c r="L686" t="inlineStr"/>
@@ -39603,7 +40275,11 @@
       <c r="F687" t="inlineStr"/>
       <c r="G687" t="inlineStr"/>
       <c r="H687" t="inlineStr"/>
-      <c r="I687" t="inlineStr"/>
+      <c r="I687" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J687" t="inlineStr"/>
       <c r="K687" t="inlineStr"/>
       <c r="L687" t="inlineStr"/>
@@ -39658,7 +40334,11 @@
       <c r="F688" t="inlineStr"/>
       <c r="G688" t="inlineStr"/>
       <c r="H688" t="inlineStr"/>
-      <c r="I688" t="inlineStr"/>
+      <c r="I688" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J688" t="inlineStr"/>
       <c r="K688" t="inlineStr"/>
       <c r="L688" t="inlineStr"/>
@@ -39780,7 +40460,11 @@
       <c r="F690" t="inlineStr"/>
       <c r="G690" t="inlineStr"/>
       <c r="H690" t="inlineStr"/>
-      <c r="I690" t="inlineStr"/>
+      <c r="I690" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J690" t="inlineStr"/>
       <c r="K690" t="inlineStr"/>
       <c r="L690" t="inlineStr"/>
@@ -40024,7 +40708,11 @@
       <c r="F694" t="inlineStr"/>
       <c r="G694" t="inlineStr"/>
       <c r="H694" t="inlineStr"/>
-      <c r="I694" t="inlineStr"/>
+      <c r="I694" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J694" t="inlineStr"/>
       <c r="K694" t="inlineStr"/>
       <c r="L694" t="inlineStr"/>
@@ -40468,7 +41156,11 @@
       <c r="F702" t="inlineStr"/>
       <c r="G702" t="inlineStr"/>
       <c r="H702" t="inlineStr"/>
-      <c r="I702" t="inlineStr"/>
+      <c r="I702" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J702" t="inlineStr"/>
       <c r="K702" t="inlineStr"/>
       <c r="L702" t="inlineStr"/>
@@ -40802,7 +41494,11 @@
       <c r="F708" t="inlineStr"/>
       <c r="G708" t="inlineStr"/>
       <c r="H708" t="inlineStr"/>
-      <c r="I708" t="inlineStr"/>
+      <c r="I708" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J708" t="inlineStr"/>
       <c r="K708" t="inlineStr"/>
       <c r="L708" t="inlineStr"/>
@@ -40918,7 +41614,7 @@
       <c r="H710" t="inlineStr"/>
       <c r="I710" t="inlineStr">
         <is>
-          <t>Middle Eastern/Arab</t>
+          <t>Black/African</t>
         </is>
       </c>
       <c r="J710" t="inlineStr"/>
@@ -41144,7 +41840,11 @@
       <c r="F714" t="inlineStr"/>
       <c r="G714" t="inlineStr"/>
       <c r="H714" t="inlineStr"/>
-      <c r="I714" t="inlineStr"/>
+      <c r="I714" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J714" t="inlineStr"/>
       <c r="K714" t="inlineStr"/>
       <c r="L714" t="inlineStr"/>
@@ -41199,7 +41899,11 @@
       <c r="F715" t="inlineStr"/>
       <c r="G715" t="inlineStr"/>
       <c r="H715" t="inlineStr"/>
-      <c r="I715" t="inlineStr"/>
+      <c r="I715" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J715" t="inlineStr"/>
       <c r="K715" t="inlineStr"/>
       <c r="L715" t="inlineStr"/>
@@ -41256,7 +41960,7 @@
       <c r="H716" t="inlineStr"/>
       <c r="I716" t="inlineStr">
         <is>
-          <t>Black/African</t>
+          <t>East/SE Asian</t>
         </is>
       </c>
       <c r="J716" t="inlineStr"/>
@@ -41368,7 +42072,11 @@
       <c r="F718" t="inlineStr"/>
       <c r="G718" t="inlineStr"/>
       <c r="H718" t="inlineStr"/>
-      <c r="I718" t="inlineStr"/>
+      <c r="I718" t="inlineStr">
+        <is>
+          <t>Middle Eastern/Arab</t>
+        </is>
+      </c>
       <c r="J718" t="inlineStr"/>
       <c r="K718" t="inlineStr"/>
       <c r="L718" t="inlineStr"/>
@@ -41425,7 +42133,7 @@
       <c r="H719" t="inlineStr"/>
       <c r="I719" t="inlineStr">
         <is>
-          <t>Middle Eastern/Arab</t>
+          <t>South Asian</t>
         </is>
       </c>
       <c r="J719" t="inlineStr"/>
@@ -41482,7 +42190,11 @@
       <c r="F720" t="inlineStr"/>
       <c r="G720" t="inlineStr"/>
       <c r="H720" t="inlineStr"/>
-      <c r="I720" t="inlineStr"/>
+      <c r="I720" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J720" t="inlineStr"/>
       <c r="K720" t="inlineStr"/>
       <c r="L720" t="inlineStr"/>
@@ -41649,7 +42361,7 @@
       <c r="H723" t="inlineStr"/>
       <c r="I723" t="inlineStr">
         <is>
-          <t>Hispanic/Latino</t>
+          <t>South Asian</t>
         </is>
       </c>
       <c r="J723" t="inlineStr"/>
@@ -41816,7 +42528,11 @@
       <c r="F726" t="inlineStr"/>
       <c r="G726" t="inlineStr"/>
       <c r="H726" t="inlineStr"/>
-      <c r="I726" t="inlineStr"/>
+      <c r="I726" t="inlineStr">
+        <is>
+          <t>Middle Eastern/Arab</t>
+        </is>
+      </c>
       <c r="J726" t="inlineStr"/>
       <c r="K726" t="inlineStr"/>
       <c r="L726" t="inlineStr"/>
@@ -42335,7 +43051,11 @@
       <c r="F735" t="inlineStr"/>
       <c r="G735" t="inlineStr"/>
       <c r="H735" t="inlineStr"/>
-      <c r="I735" t="inlineStr"/>
+      <c r="I735" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J735" t="inlineStr"/>
       <c r="K735" t="inlineStr"/>
       <c r="L735" t="inlineStr"/>
@@ -42669,7 +43389,11 @@
       <c r="F741" t="inlineStr"/>
       <c r="G741" t="inlineStr"/>
       <c r="H741" t="inlineStr"/>
-      <c r="I741" t="inlineStr"/>
+      <c r="I741" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J741" t="inlineStr"/>
       <c r="K741" t="inlineStr"/>
       <c r="L741" t="inlineStr"/>
@@ -44516,7 +45240,11 @@
       <c r="F774" t="inlineStr"/>
       <c r="G774" t="inlineStr"/>
       <c r="H774" t="inlineStr"/>
-      <c r="I774" t="inlineStr"/>
+      <c r="I774" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J774" t="inlineStr"/>
       <c r="K774" t="inlineStr"/>
       <c r="L774" t="inlineStr"/>
@@ -44626,7 +45354,11 @@
       <c r="F776" t="inlineStr"/>
       <c r="G776" t="inlineStr"/>
       <c r="H776" t="inlineStr"/>
-      <c r="I776" t="inlineStr"/>
+      <c r="I776" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J776" t="inlineStr"/>
       <c r="K776" t="inlineStr"/>
       <c r="L776" t="inlineStr"/>
@@ -45074,7 +45806,11 @@
       <c r="F784" t="inlineStr"/>
       <c r="G784" t="inlineStr"/>
       <c r="H784" t="inlineStr"/>
-      <c r="I784" t="inlineStr"/>
+      <c r="I784" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J784" t="inlineStr"/>
       <c r="K784" t="inlineStr"/>
       <c r="L784" t="inlineStr"/>
@@ -45184,7 +45920,11 @@
       <c r="F786" t="inlineStr"/>
       <c r="G786" t="inlineStr"/>
       <c r="H786" t="inlineStr"/>
-      <c r="I786" t="inlineStr"/>
+      <c r="I786" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J786" t="inlineStr"/>
       <c r="K786" t="inlineStr"/>
       <c r="L786" t="inlineStr"/>
@@ -45294,7 +46034,11 @@
       <c r="F788" t="inlineStr"/>
       <c r="G788" t="inlineStr"/>
       <c r="H788" t="inlineStr"/>
-      <c r="I788" t="inlineStr"/>
+      <c r="I788" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J788" t="inlineStr"/>
       <c r="K788" t="inlineStr"/>
       <c r="L788" t="inlineStr"/>
@@ -45349,7 +46093,11 @@
       <c r="F789" t="inlineStr"/>
       <c r="G789" t="inlineStr"/>
       <c r="H789" t="inlineStr"/>
-      <c r="I789" t="inlineStr"/>
+      <c r="I789" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J789" t="inlineStr"/>
       <c r="K789" t="inlineStr"/>
       <c r="L789" t="inlineStr"/>
@@ -45463,7 +46211,11 @@
       <c r="F791" t="inlineStr"/>
       <c r="G791" t="inlineStr"/>
       <c r="H791" t="inlineStr"/>
-      <c r="I791" t="inlineStr"/>
+      <c r="I791" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J791" t="inlineStr"/>
       <c r="K791" t="inlineStr"/>
       <c r="L791" t="inlineStr"/>
@@ -45518,7 +46270,11 @@
       <c r="F792" t="inlineStr"/>
       <c r="G792" t="inlineStr"/>
       <c r="H792" t="inlineStr"/>
-      <c r="I792" t="inlineStr"/>
+      <c r="I792" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J792" t="inlineStr"/>
       <c r="K792" t="inlineStr"/>
       <c r="L792" t="inlineStr"/>
@@ -46139,7 +46895,11 @@
       <c r="F803" t="inlineStr"/>
       <c r="G803" t="inlineStr"/>
       <c r="H803" t="inlineStr"/>
-      <c r="I803" t="inlineStr"/>
+      <c r="I803" t="inlineStr">
+        <is>
+          <t>White/European</t>
+        </is>
+      </c>
       <c r="J803" t="inlineStr"/>
       <c r="K803" t="inlineStr"/>
       <c r="L803" t="inlineStr"/>
@@ -46249,7 +47009,11 @@
       <c r="F805" t="inlineStr"/>
       <c r="G805" t="inlineStr"/>
       <c r="H805" t="inlineStr"/>
-      <c r="I805" t="inlineStr"/>
+      <c r="I805" t="inlineStr">
+        <is>
+          <t>South Asian</t>
+        </is>
+      </c>
       <c r="J805" t="inlineStr"/>
       <c r="K805" t="inlineStr"/>
       <c r="L805" t="inlineStr"/>
@@ -46377,7 +47141,7 @@
       <c r="H807" t="inlineStr"/>
       <c r="I807" t="inlineStr">
         <is>
-          <t>Middle Eastern/Arab</t>
+          <t>South Asian</t>
         </is>
       </c>
       <c r="J807" t="inlineStr"/>
@@ -46544,7 +47308,11 @@
       <c r="F810" t="inlineStr"/>
       <c r="G810" t="inlineStr"/>
       <c r="H810" t="inlineStr"/>
-      <c r="I810" t="inlineStr"/>
+      <c r="I810" t="inlineStr">
+        <is>
+          <t>Black/African</t>
+        </is>
+      </c>
       <c r="J810" t="inlineStr"/>
       <c r="K810" t="inlineStr"/>
       <c r="L810" t="inlineStr"/>
@@ -46725,7 +47493,11 @@
       <c r="F813" t="inlineStr"/>
       <c r="G813" t="inlineStr"/>
       <c r="H813" t="inlineStr"/>
-      <c r="I813" t="inlineStr"/>
+      <c r="I813" t="inlineStr">
+        <is>
+          <t>South Asian</t>
+        </is>
+      </c>
       <c r="J813" t="inlineStr"/>
       <c r="K813" t="inlineStr"/>
       <c r="L813" t="inlineStr"/>
@@ -46780,7 +47552,11 @@
       <c r="F814" t="inlineStr"/>
       <c r="G814" t="inlineStr"/>
       <c r="H814" t="inlineStr"/>
-      <c r="I814" t="inlineStr"/>
+      <c r="I814" t="inlineStr">
+        <is>
+          <t>Middle Eastern/Arab</t>
+        </is>
+      </c>
       <c r="J814" t="inlineStr"/>
       <c r="K814" t="inlineStr"/>
       <c r="L814" t="inlineStr"/>

</xml_diff>